<commit_message>
fix(inventario): fixture mixto.xlsx sin la columna Costo total
325aa378 quito la columna de la importacion pero el fixture del lector .xlsx
la seguia trayendo, y tests/integration/inventario/xlsx-reader.test.ts caia
con unknown_columns. Se quita la columna H del fixture (Lote..Alerta se
desplazan) y el decimal nativo 100.25 pasa a Costo unitario.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/inventario-importar/mixto.xlsx
+++ b/tests/fixtures/inventario-importar/mixto.xlsx
@@ -466,10 +466,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A44B9664-9C43-449C-9079-08EFD0270549}">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -492,22 +492,19 @@
         <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
@@ -523,20 +520,20 @@
       <c r="G2">
         <v>3.5</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J2" s="2">
+      <c r="I2" s="2">
         <v>46037</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="L2">
+      <c r="K2">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -552,20 +549,20 @@
       <c r="G3">
         <v>1E-4</v>
       </c>
+      <c r="H3" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="I3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="J3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="2">
+      <c r="J3" s="2">
         <v>46568</v>
       </c>
-      <c r="L3">
+      <c r="K3">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
@@ -578,10 +575,10 @@
       <c r="F5">
         <v>1234567</v>
       </c>
-      <c r="H5">
+      <c r="G5">
         <v>100.25</v>
       </c>
-      <c r="L5">
+      <c r="K5">
         <v>10</v>
       </c>
     </row>

</xml_diff>